<commit_message>
Suppression du profil FHIR FRMedicationsCombinaison (#132) 43b87997e2d0d33029bf4a25810de22c452f6d87
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-care-plan-document.xlsx
+++ b/main/ig/StructureDefinition-fr-care-plan-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-23T15:25:59+00:00</t>
+    <t>2026-05-06T07:44:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1603,7 +1603,7 @@
   </si>
   <si>
     <t>CodeableConcept
-Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-medication-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-medications-combinaison-document)</t>
+Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-medication-document)</t>
   </si>
   <si>
     <t>Produit de santé</t>
@@ -2019,7 +2019,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="167.2421875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="126.609375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>